<commit_message>
Flor Alpuy Update Showroom Preventa 2026 2026-10-21 17:47:41
</commit_message>
<xml_diff>
--- a/Brief Site Estrategia.xlsx
+++ b/Brief Site Estrategia.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Unidades compartidas\Gestion Comercial\1. Estrategias\2026\Navidad\Site Preventa Navidad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16731C92-11B2-4328-8B2A-30F45C5D71B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{857E8299-505A-4310-9CB4-2B3C5AC8FEC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -284,6 +284,7 @@
       <name val="Montserrat"/>
     </font>
     <font>
+      <b/>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
@@ -370,7 +371,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -416,6 +417,9 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -790,16 +794,16 @@
       <c r="A2" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="24">
         <v>282848</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="24" t="s">
         <v>48</v>
       </c>
-      <c r="D2" s="8">
+      <c r="D2" s="25">
         <v>274188</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="7" t="s">
         <v>48</v>
       </c>
       <c r="F2" s="11"/>
@@ -811,16 +815,16 @@
       <c r="A3" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="24">
         <v>282835</v>
       </c>
       <c r="C3" s="24" t="s">
         <v>50</v>
       </c>
-      <c r="D3" s="8">
+      <c r="D3" s="25">
         <v>281659</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" s="7" t="s">
         <v>49</v>
       </c>
       <c r="F3" s="9"/>

</xml_diff>

<commit_message>
Flor Alpuy Update Showroom Preventa 2026 2026-10-21 17:51:33
</commit_message>
<xml_diff>
--- a/Brief Site Estrategia.xlsx
+++ b/Brief Site Estrategia.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Unidades compartidas\Gestion Comercial\1. Estrategias\2026\Navidad\Site Preventa Navidad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{857E8299-505A-4310-9CB4-2B3C5AC8FEC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9AB1611-A3B4-4D07-A95E-DAE825F29A17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="52">
   <si>
     <t>Marca</t>
   </si>
@@ -194,6 +194,9 @@
   </si>
   <si>
     <t>Regalo Preventa - Almendras glaseadas</t>
+  </si>
+  <si>
+    <t>Regalo Preventa - Paz y humor jb + pf + gel</t>
   </si>
 </sst>
 </file>
@@ -371,7 +374,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -417,7 +420,8 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -794,13 +798,13 @@
       <c r="A2" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B2" s="24">
+      <c r="B2" s="25">
         <v>282848</v>
       </c>
       <c r="C2" s="24" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
-      <c r="D2" s="25">
+      <c r="D2" s="26">
         <v>274188</v>
       </c>
       <c r="E2" s="7" t="s">
@@ -815,13 +819,13 @@
       <c r="A3" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B3" s="24">
+      <c r="B3" s="25">
         <v>282835</v>
       </c>
       <c r="C3" s="24" t="s">
         <v>50</v>
       </c>
-      <c r="D3" s="25">
+      <c r="D3" s="26">
         <v>281659</v>
       </c>
       <c r="E3" s="7" t="s">

</xml_diff>

<commit_message>
Flor Alpuy Update Showroom Preventa 2026 2026-10-21 18:40:14
</commit_message>
<xml_diff>
--- a/Brief Site Estrategia.xlsx
+++ b/Brief Site Estrategia.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Unidades compartidas\Gestion Comercial\1. Estrategias\2026\Navidad\Site Preventa Navidad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9AB1611-A3B4-4D07-A95E-DAE825F29A17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50B7448A-0625-40DF-8F8A-BFC975B4B3DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="54">
   <si>
     <t>Marca</t>
   </si>
@@ -197,6 +197,12 @@
   </si>
   <si>
     <t>Regalo Preventa - Paz y humor jb + pf + gel</t>
+  </si>
+  <si>
+    <t>Essencial perfume + manos</t>
+  </si>
+  <si>
+    <t>Regalo essencial</t>
   </si>
 </sst>
 </file>
@@ -805,7 +811,7 @@
         <v>51</v>
       </c>
       <c r="D2" s="26">
-        <v>274188</v>
+        <v>281675</v>
       </c>
       <c r="E2" s="7" t="s">
         <v>48</v>
@@ -837,11 +843,21 @@
       <c r="I3" s="9"/>
     </row>
     <row r="4" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="7"/>
-      <c r="B4" s="8"/>
-      <c r="C4" s="9"/>
-      <c r="D4" s="10"/>
-      <c r="E4" s="11"/>
+      <c r="A4" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4" s="8">
+        <v>282836</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="D4" s="10">
+        <v>281677</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>53</v>
+      </c>
       <c r="F4" s="11"/>
       <c r="G4" s="11"/>
       <c r="H4" s="11"/>

</xml_diff>